<commit_message>
Add SOC - vælgSmiley
</commit_message>
<xml_diff>
--- a/Use Case.xlsx
+++ b/Use Case.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Datamatiker\Projekter\Hydac\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Itzar\Desktop\Datamatiker\Git\HYDAC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB5BB8D8-FF5E-4456-B0A0-90F19AFBD58E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D549EB0A-4254-4FF5-A4AD-3D8F731443CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="561" xr2:uid="{FAE73960-6D5B-49EE-8D5E-7E75CD0D9398}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="561" xr2:uid="{FAE73960-6D5B-49EE-8D5E-7E75CD0D9398}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="70">
   <si>
     <t>Primær aktør</t>
   </si>
@@ -104,9 +104,6 @@
     <t>10. Systemet skriver "God dag" og timerne bliver registreret til lønafdelingen</t>
   </si>
   <si>
-    <t>Medarbejder booker møde med kunde</t>
-  </si>
-  <si>
     <t>Bruger system til at booke møde</t>
   </si>
   <si>
@@ -146,46 +143,112 @@
     <t xml:space="preserve">Medarbejder </t>
   </si>
   <si>
-    <t>Tjek ind og ud</t>
-  </si>
-  <si>
     <t>Tjekker ind om morgenen, og ud efter arbejde</t>
   </si>
   <si>
     <t>Registrere sin ankomst, og melde sin afgang</t>
   </si>
   <si>
-    <t>Besøgende</t>
-  </si>
-  <si>
     <t>Bruger system til at melde ankomst</t>
   </si>
   <si>
     <t>Registrere besøgende er klar til møde</t>
   </si>
   <si>
-    <t>1.Besøgende ankommer til firma</t>
-  </si>
-  <si>
-    <t>2. Besøgende går op til skærm</t>
-  </si>
-  <si>
-    <t>3. Besøgende vælger "Gæst"</t>
-  </si>
-  <si>
-    <t>4. Besøgende vælger "Meld ankomst"</t>
-  </si>
-  <si>
-    <t>5. System spørger om navn og firma navn</t>
-  </si>
-  <si>
-    <t>6. Besøgende indtaster oplysninger</t>
-  </si>
-  <si>
     <t>7. Systemet registrerer ankomst, og skriver "Ankomst registreret"</t>
   </si>
   <si>
     <t>8. Systemet giver reception? Besked, og ansvarlige for møde bliver advaret.</t>
+  </si>
+  <si>
+    <t>Se hvem der er på arbejde</t>
+  </si>
+  <si>
+    <t>Medarbejder slår op hvem der er tjekket ind</t>
+  </si>
+  <si>
+    <t>Få overblik over hvem der er til stede</t>
+  </si>
+  <si>
+    <t>3. Medarbejder indtaster sit personlige 4-cifrede mearbejdernummer</t>
+  </si>
+  <si>
+    <t>4. Medarbejder vælger "Se tilstedeværelse"</t>
+  </si>
+  <si>
+    <t>5. Systemet henter alle medarbejdere, der er tjekket ind.</t>
+  </si>
+  <si>
+    <t>6. Systemet viser listen med medarbejdernes navne og valgte smileys.</t>
+  </si>
+  <si>
+    <t>7. Medarbejder finder den ønskede kollega på listen</t>
+  </si>
+  <si>
+    <t>UC4</t>
+  </si>
+  <si>
+    <t>Bookning af mødelokale</t>
+  </si>
+  <si>
+    <t>UC5</t>
+  </si>
+  <si>
+    <t>Gæst</t>
+  </si>
+  <si>
+    <t>1. Gæst går hen til skærmen</t>
+  </si>
+  <si>
+    <t>2. Gæst vælger "Gæst"</t>
+  </si>
+  <si>
+    <t>3. Gæst indtaster sit eget navn</t>
+  </si>
+  <si>
+    <t>4. Systemet slår op, hvilket medarbejder gæsten er tilknyttet</t>
+  </si>
+  <si>
+    <t>5. Systemet tjekker om gæsten har en aftale med deres tilknyttede kontaktperson</t>
+  </si>
+  <si>
+    <t>Tjekker ind til aftale med kontaktperson</t>
+  </si>
+  <si>
+    <t>Registrere sin ankomst, og få detaljer om mødet</t>
+  </si>
+  <si>
+    <t>6. Systemet registrere gæstens ankomsttidspunkt</t>
+  </si>
+  <si>
+    <t>7. Systemet viser den tilrettelagte "mødelokale" og "tidsperiode" for mødet</t>
+  </si>
+  <si>
+    <t>8. Skærmen viser "Tjek ind bekræftet, Velkommen til HYDAC!"</t>
+  </si>
+  <si>
+    <t>1.Gæst ankommer til firma</t>
+  </si>
+  <si>
+    <t>2. Gæst går op til skærm</t>
+  </si>
+  <si>
+    <t>3. Gæst vælger "Gæst"</t>
+  </si>
+  <si>
+    <t>4. Gæst vælger "Meld ankomst"</t>
+  </si>
+  <si>
+    <t>5. Gæst spørger om navn og firma navn</t>
+  </si>
+  <si>
+    <t>6. Gæst indtaster oplysninger</t>
+  </si>
+  <si>
+    <t>Tjek ind til konsultation</t>
+  </si>
+  <si>
+    <t>Tjek ind og ud for arbejde</t>
   </si>
 </sst>
 </file>
@@ -235,12 +298,12 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="20" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -259,7 +322,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -575,272 +638,454 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39673B22-004F-4717-8A37-72698BEC2F7D}">
-  <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:H35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="59.53125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="63.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="63.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="59.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="63.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="63.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="D1" s="1" t="s">
+      <c r="B1" s="3"/>
+      <c r="D1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1"/>
-      <c r="G1" s="1" t="s">
+      <c r="E1" s="3"/>
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
+      <c r="H1" s="3"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A3" s="2" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" s="1"/>
+      <c r="H8" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="1"/>
+      <c r="H9" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="1"/>
+      <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="1"/>
+      <c r="H10" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="1"/>
+      <c r="B11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="1"/>
+      <c r="H11" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="1"/>
+      <c r="B12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G12" s="1"/>
+      <c r="H12" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="1"/>
+      <c r="B13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="1"/>
+      <c r="H13" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" s="1"/>
+      <c r="B14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G14" s="1"/>
+      <c r="H14" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="1"/>
+      <c r="B15" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" s="1"/>
+      <c r="B16" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="1"/>
+      <c r="B17" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="D19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="B21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3" s="3" t="s">
+      <c r="E21" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A4" s="2" t="s">
+      <c r="D22" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A5" s="2" t="s">
+      <c r="E22" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="B23" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A6" s="2" t="s">
+      <c r="E23" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="B24" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E24" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="1"/>
+      <c r="B26" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A8" s="2"/>
-      <c r="B8" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G9" s="2"/>
-      <c r="H9" s="3" t="s">
+      <c r="D26" s="1"/>
+      <c r="E26" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="1"/>
+      <c r="B27" s="4" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="3" t="s">
+      <c r="D27" s="1"/>
+      <c r="E27" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" s="1"/>
+      <c r="B28" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="3" t="s">
+      <c r="D28" s="1"/>
+      <c r="E28" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" s="1"/>
+      <c r="B29" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A12" s="2"/>
-      <c r="B12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="3" t="s">
+      <c r="D29" s="1"/>
+      <c r="E29" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" s="1"/>
+      <c r="B30" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A13" s="2"/>
-      <c r="B13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="3" t="s">
+      <c r="D30" s="1"/>
+      <c r="E30" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" s="1"/>
+      <c r="B31" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A14" s="4"/>
-      <c r="B14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G14" s="4"/>
-      <c r="H14" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A15" s="4"/>
-      <c r="B15" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A16" s="4"/>
-      <c r="B16" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A17" s="4"/>
-      <c r="B17" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" s="1"/>
+      <c r="B32" s="2"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" s="1"/>
+      <c r="B33" s="2"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" s="1"/>
+      <c r="B34" s="2"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" s="1"/>
+      <c r="B35" s="2"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="D19:E19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>